<commit_message>
feat(parser): 支持 repeated 外键校验
</commit_message>
<xml_diff>
--- a/assets/xls/商店.xlsx
+++ b/assets/xls/商店.xlsx
@@ -4,14 +4,14 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="21315" windowHeight="10680" tabRatio="535"/>
+    <workbookView windowWidth="21555" windowHeight="11265" tabRatio="535"/>
   </bookViews>
   <sheets>
     <sheet name="Shop" sheetId="7" r:id="rId1"/>
     <sheet name="#备注" sheetId="8" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Shop!$A$4:$C$12</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Shop!$A$4:$D$12</definedName>
     <definedName name="CSpreadSheetBackup">#REF!</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
@@ -51,12 +51,25 @@
         </r>
       </text>
     </comment>
+    <comment ref="C1" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <rFont val="宋体"/>
+            <charset val="134"/>
+          </rPr>
+          <t xml:space="preserve">fk:Item.ID;
+</t>
+        </r>
+      </text>
+    </comment>
   </commentList>
 </comments>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="32">
   <si>
     <t>ID</t>
   </si>
@@ -64,6 +77,9 @@
     <t>ItemId</t>
   </si>
   <si>
+    <t>ItemList</t>
+  </si>
+  <si>
     <t>ItemName</t>
   </si>
   <si>
@@ -76,6 +92,9 @@
     <t>int32</t>
   </si>
   <si>
+    <t>repeated int32</t>
+  </si>
+  <si>
     <t>string</t>
   </si>
   <si>
@@ -94,28 +113,52 @@
     <t>售价</t>
   </si>
   <si>
+    <t>8;9</t>
+  </si>
+  <si>
     <t>点券</t>
   </si>
   <si>
+    <t>9;10</t>
+  </si>
+  <si>
     <t>经验</t>
   </si>
   <si>
+    <t>10;11</t>
+  </si>
+  <si>
     <t>金币</t>
   </si>
   <si>
+    <t>11;12</t>
+  </si>
+  <si>
     <t>钻石</t>
   </si>
   <si>
+    <t>12;13</t>
+  </si>
+  <si>
     <t>积分</t>
   </si>
   <si>
+    <t>13;14</t>
+  </si>
+  <si>
     <t>徽章</t>
   </si>
   <si>
+    <t>14;15</t>
+  </si>
+  <si>
     <t>龙鳞</t>
   </si>
   <si>
     <t>999999999999</t>
+  </si>
+  <si>
+    <t>15;14</t>
   </si>
   <si>
     <t>植物碎片</t>
@@ -1122,17 +1165,18 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:D12"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.25" outlineLevelCol="3"/>
+  <dimension ref="A1:E12"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.25" outlineLevelCol="4"/>
   <cols>
     <col min="1" max="1" width="10.375" style="2" customWidth="1"/>
-    <col min="2" max="2" width="9.375" style="2" customWidth="1"/>
-    <col min="3" max="3" width="10.375" style="2" customWidth="1"/>
-    <col min="4" max="4" width="14.875" style="2" customWidth="1"/>
-    <col min="5" max="16384" width="9" style="2"/>
+    <col min="2" max="2" width="8.125" style="2" customWidth="1"/>
+    <col min="3" max="3" width="17.875" style="2" customWidth="1"/>
+    <col min="4" max="4" width="10.375" style="2" customWidth="1"/>
+    <col min="5" max="5" width="14.875" style="2" customWidth="1"/>
+    <col min="6" max="16384" width="9" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" s="1" customFormat="1" spans="1:4">
+    <row r="1" s="1" customFormat="1" spans="1:5">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1145,48 +1189,60 @@
       <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
     </row>
-    <row r="2" s="1" customFormat="1" spans="1:4">
+    <row r="2" s="1" customFormat="1" spans="1:5">
       <c r="A2" s="1" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>9</v>
       </c>
     </row>
-    <row r="3" s="1" customFormat="1" spans="1:4">
+    <row r="3" s="1" customFormat="1" spans="1:5">
       <c r="A3" s="1" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C3" s="1"/>
-      <c r="D3" s="1" t="s">
-        <v>8</v>
+        <v>10</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D3" s="1"/>
+      <c r="E3" s="1" t="s">
+        <v>10</v>
       </c>
     </row>
-    <row r="4" s="1" customFormat="1" spans="1:4">
+    <row r="4" s="1" customFormat="1" spans="1:5">
       <c r="A4" s="1" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>11</v>
+        <v>12</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>13</v>
       </c>
     </row>
-    <row r="5" s="1" customFormat="1" spans="1:4">
+    <row r="5" s="1" customFormat="1" spans="1:5">
       <c r="A5" s="2">
         <v>1</v>
       </c>
@@ -1194,13 +1250,16 @@
         <v>8</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="D5" s="3">
+        <v>14</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="E5" s="3">
         <v>10</v>
       </c>
     </row>
-    <row r="6" spans="1:4">
+    <row r="6" spans="1:5">
       <c r="A6" s="2">
         <v>2</v>
       </c>
@@ -1208,13 +1267,16 @@
         <v>9</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="D6" s="3">
+        <v>16</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="E6" s="3">
         <v>1000</v>
       </c>
     </row>
-    <row r="7" spans="1:4">
+    <row r="7" spans="1:5">
       <c r="A7" s="2">
         <v>3</v>
       </c>
@@ -1222,13 +1284,16 @@
         <v>10</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="D7" s="3">
+        <v>18</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="E7" s="3">
         <v>10000</v>
       </c>
     </row>
-    <row r="8" spans="1:4">
+    <row r="8" spans="1:5">
       <c r="A8" s="2">
         <v>4</v>
       </c>
@@ -1236,13 +1301,16 @@
         <v>11</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="D8" s="3">
+        <v>20</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="E8" s="3">
         <v>100000000</v>
       </c>
     </row>
-    <row r="9" spans="1:4">
+    <row r="9" spans="1:5">
       <c r="A9" s="2">
         <v>5</v>
       </c>
@@ -1250,13 +1318,16 @@
         <v>12</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="D9" s="3">
+        <v>22</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="E9" s="3">
         <v>999999999</v>
       </c>
     </row>
-    <row r="10" spans="1:4">
+    <row r="10" spans="1:5">
       <c r="A10" s="2">
         <v>6</v>
       </c>
@@ -1264,13 +1335,16 @@
         <v>13</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="D10" s="3">
+        <v>24</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="E10" s="3">
         <v>99999999999</v>
       </c>
     </row>
-    <row r="11" spans="1:4">
+    <row r="11" spans="1:5">
       <c r="A11" s="2">
         <v>7</v>
       </c>
@@ -1278,13 +1352,16 @@
         <v>14</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="D11" s="4" t="s">
-        <v>19</v>
+        <v>26</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="E11" s="4" t="s">
+        <v>28</v>
       </c>
     </row>
-    <row r="12" spans="1:4">
+    <row r="12" spans="1:5">
       <c r="A12" s="2">
         <v>8</v>
       </c>
@@ -1292,17 +1369,20 @@
         <v>15</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="D12" s="4" t="s">
-        <v>21</v>
+        <v>29</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="E12" s="4" t="s">
+        <v>31</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>
   <ignoredErrors>
-    <ignoredError sqref="D5:D12" numberStoredAsText="1"/>
+    <ignoredError sqref="E5:E12" numberStoredAsText="1"/>
   </ignoredErrors>
   <legacyDrawing r:id="rId2"/>
 </worksheet>

</xml_diff>